<commit_message>
use abstract class to re-code and make fast
</commit_message>
<xml_diff>
--- a/P2Dmodel/OCP/OCP_from_COMSOL.xlsx
+++ b/P2Dmodel/OCP/OCP_from_COMSOL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailscuteducn-my.sharepoint.com/personal/202110182474_mail_scut_edu_cn/Documents/代码/电池模型/P2Dmodel/OCP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailscuteducn-my.sharepoint.com/personal/202110182474_mail_scut_edu_cn/Documents/Code/Battery/P2Dmodel/OCP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{D18E3EAD-39EA-4CFB-A650-8A43D183F7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C6406AF-665A-4AE2-A36F-192BACC0D5E4}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{D18E3EAD-39EA-4CFB-A650-8A43D183F7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2361DFAE-BFC6-411B-A96F-B05BCB340027}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,17 +35,17 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="4">
   <si>
-    <t>OCP</t>
+    <t>θs</t>
   </si>
   <si>
-    <t>OCP</t>
+    <t>θs</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>θ</t>
+    <t>UOCP</t>
   </si>
   <si>
-    <t>θ</t>
+    <t>UOCP</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -376,10 +376,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>3</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1188,10 +1188,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1927,10 +1927,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -2443,10 +2443,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -2658,10 +2658,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3013,10 +3013,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3160,10 +3160,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3483,10 +3483,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3838,10 +3838,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>